<commit_message>
Agrega graficos nativos interactivos de dispersion y barras en la exportacion de Excel
</commit_message>
<xml_diff>
--- a/analisis_micmac_convergente.xlsx
+++ b/analisis_micmac_convergente.xlsx
@@ -18,6 +18,7 @@
     <sheet name="9_Flujos_Netos_Indirectos" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="10_Indicadores_4D" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="11_Diagnostico_Prospectivo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="12_Graficos_Estructurales" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -315,6 +316,872 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Plano Dinámico (Motricidad Neta vs. Dependencia Neta)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="9"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'10_Indicadores_4D'!$F$5:$F$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'10_Indicadores_4D'!$E$5:$E$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Dependencia Neta (Dⁿᵉᵗᵃ)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Motricidad Neta (Mⁿᵉᵗᵃ)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Desplazamiento: Motricidad Clásica vs. Neta Dinámica</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$B$5:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$E$5:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Variable</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Intensidad Motriz</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>1. Plano Estructural Dinámico 4D (Motricidad Neta vs. Dependencia Neta)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="10"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'10_Indicadores_4D'!$F$5:$F$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'10_Indicadores_4D'!$E$5:$E$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Dependencia Neta Efectiva</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Motricidad Neta Efectiva</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>2. Comparativa: Motricidad Clásica (Godet) vs. Neta (Katz-Bonacich)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$B$5:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$E$5:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Variable</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Intensidad de Motricidad</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="11"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>3. Retorno Sistémico / Bucle Propio F (+ Amplificador / − Regulador)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!I4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$I$5:$I$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Variable</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Valor Bucle F</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>4. Índice de Ambigüedad y Contradicción Estructural Ω (%)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'10_Indicadores_4D'!J4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'10_Indicadores_4D'!$A$5:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'10_Indicadores_4D'!$J$5:$J$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Variable</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Contradicción Sistémica (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>14</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>14</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1386,6 +2253,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1658,6 +2526,35 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TABLERO DE GRÁFICOS ESTRUCTURALES Y PROSPECTIVOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Visualizaciones nativas interactivas en Excel: planos de cuadrantes, desplazamientos de motricidad, bucles propios y contradicción.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Agregar numero correlativo N° a las variables en tablas, matriz y reportes
</commit_message>
<xml_diff>
--- a/analisis_micmac_convergente.xlsx
+++ b/analisis_micmac_convergente.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_Base_Variables" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_Base_Matriz_Directa" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_Base_Justificaciones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_Matriz_A_Polaridad" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5_Matriz_T_Retardos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6_Matriz_W_Efectiva" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7_Matriz_S_Bruta_Leontief" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8_Matriz_S_Neta_Leontief" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9_Flujos_Netos_Indirectos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10_Indicadores_4D" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11_Diagnostico_Prospectivo" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="12_Graficos_Estructurales" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Base_Variables" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Base_Matriz_Directa" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Base_Justificaciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Matriz_A_Polaridad" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Matriz_T_Retardos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Matriz_W_Efectiva" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Matriz_S_Bruta_Leontief" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Matriz_S_Neta_Leontief" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Flujos_Netos_Indirectos" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Indicadores_4D" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Diagnostico_Prospectivo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Graficos_Estructurales" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -319,14 +319,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -343,7 +343,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -352,7 +352,7 @@
             <symbol val="circle"/>
             <size val="9"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -381,8 +381,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -407,8 +407,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -434,14 +434,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -465,7 +465,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -489,7 +489,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -517,8 +517,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -544,8 +544,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -571,14 +571,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -595,7 +595,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -604,7 +604,7 @@
             <symbol val="circle"/>
             <size val="10"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -633,8 +633,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -659,8 +659,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -686,14 +686,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -717,7 +717,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -741,7 +741,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -769,8 +769,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -796,8 +796,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -823,14 +823,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="11"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -854,7 +854,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -882,8 +882,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -909,8 +909,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -933,14 +933,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -964,7 +964,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -992,8 +992,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1019,8 +1019,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1043,7 +1043,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>14</col>
@@ -1058,9 +1058,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1080,9 +1080,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1092,7 +1092,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1107,9 +1107,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1129,9 +1129,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1151,9 +1151,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1173,9 +1173,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1473,13 +1473,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="93" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="93" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1500,202 +1501,234 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Nombre de la Variable</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Definición y Alcance Conceptual</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Valor Inicial (x₀)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>LID</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Liderazgo directivo</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Capacidad de la dirección de fijar prioridades, patrocinar proyectos y comunicar el rumbo.</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="E5" s="7" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>INV</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Inversión y presupuesto</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Recursos económicos disponibles para tecnología, formación y mantenimiento.</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="E6" s="7" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>INF</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Infraestructura tecnológica</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Plataformas, conectividad, equipos y soporte técnico.</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="E7" s="7" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>COM</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Competencias docentes</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Dominio pedagógico y digital del cuerpo docente.</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="E8" s="7" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>CUL</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Cultura de innovación</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Disposición colectiva a experimentar, compartir y aprender de errores.</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="E9" s="7" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>EXP</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Experiencia estudiantil</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Calidad percibida del aprendizaje y de los servicios.</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="E10" s="7" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>RES</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Resistencia al cambio</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Oposición activa o pasiva a nuevas formas de trabajo.</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="E11" s="7" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>RET</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Retención estudiantil</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Proporción de estudiantes que continúan sus estudios.</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="E12" s="7" t="n">
         <v>55</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>NOR</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Normativa y acreditación</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Exigencias externas de calidad y regulación (variable exógena).</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="E13" s="7" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1710,22 +1743,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="65" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="65" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1746,506 +1780,538 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Motricidad Clásica</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>Dependencia Clásica</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>Rango Clásico</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="F4" s="27" t="inlineStr">
         <is>
           <t>Motricidad Neta</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="G4" s="27" t="inlineStr">
         <is>
           <t>Dependencia Neta</t>
         </is>
       </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="H4" s="27" t="inlineStr">
         <is>
           <t>Rango Dinámico</t>
         </is>
       </c>
-      <c r="H4" s="27" t="inlineStr">
+      <c r="I4" s="27" t="inlineStr">
         <is>
           <t>Δ Rango</t>
         </is>
       </c>
-      <c r="I4" s="27" t="inlineStr">
+      <c r="J4" s="27" t="inlineStr">
         <is>
           <t>Bucle Propio (F)</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="K4" s="27" t="inlineStr">
         <is>
           <t>Ambigüedad Ω (%)</t>
         </is>
       </c>
-      <c r="K4" s="27" t="inlineStr">
+      <c r="L4" s="27" t="inlineStr">
         <is>
           <t>Cuadrante Dinámico</t>
         </is>
       </c>
-      <c r="L4" s="27" t="inlineStr">
+      <c r="M4" s="27" t="inlineStr">
         <is>
           <t>Trampa de Política</t>
         </is>
       </c>
-      <c r="M4" s="27" t="inlineStr">
+      <c r="N4" s="27" t="inlineStr">
         <is>
           <t>Rol Estratégico Diagnóstico</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>LID · Liderazgo directivo</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="C5" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="D5" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="28" t="n">
-        <v>43.9492450288867</v>
-      </c>
       <c r="F5" s="28" t="n">
-        <v>9.369076831979745</v>
-      </c>
-      <c r="G5" s="4" t="n">
+        <v>43.94924502888664</v>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>9.369076831979729</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>1.46592057393983</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>3.227821707752609</v>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>Variable motriz / de entrada</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>1.465920573939827</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>3.227821707752598</v>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Variable motriz / determinante</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Palanca maestra consistente</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>INV · Inversión y presupuesto</t>
         </is>
-      </c>
-      <c r="B6" s="13" t="n">
-        <v>6</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="28" t="n">
-        <v>24.47934017483544</v>
-      </c>
       <c r="F6" s="28" t="n">
-        <v>16.01218796775074</v>
-      </c>
-      <c r="G6" s="4" t="n">
+        <v>24.4793401748354</v>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>16.01218796775072</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="29" t="n">
+      <c r="I6" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="21" t="n">
-        <v>1.418498526558171</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>5.477285355406258</v>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>Variable motriz / de entrada</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="J6" s="21" t="n">
+        <v>1.418498526558168</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>5.47728535540627</v>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Variable motriz / determinante</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Palanca maestra consistente</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>INF · Infraestructura tecnológica</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="C7" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="D7" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="28" t="n">
-        <v>21.82293547504057</v>
-      </c>
       <c r="F7" s="28" t="n">
-        <v>15.7987018760697</v>
-      </c>
-      <c r="G7" s="4" t="n">
+        <v>21.82293547504054</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>15.79870187606968</v>
+      </c>
+      <c r="H7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="I7" s="30" t="n">
         <v>-1</v>
       </c>
-      <c r="I7" s="21" t="n">
-        <v>1.170937222634377</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>5.09238803758697</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="J7" s="21" t="n">
+        <v>1.170937222634375</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>5.092388037586981</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Variable autónoma</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Palanca maestra consistente</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>COM · Competencias docentes</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="C8" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="D8" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="28" t="n">
-        <v>23.64617665946394</v>
-      </c>
       <c r="F8" s="28" t="n">
-        <v>34.27579955718877</v>
-      </c>
-      <c r="G8" s="4" t="n">
+        <v>23.6461766594639</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>34.27579955718872</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="I8" s="30" t="n">
         <v>-1</v>
       </c>
-      <c r="I8" s="21" t="n">
-        <v>3.958993217981114</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>14.34149195805466</v>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Variable de enlace / reto</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="J8" s="21" t="n">
+        <v>3.958993217981105</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>14.34149195805468</v>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Variable crítica / estratégica (enlace)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Falsa variable clave (espejismo); Nodo de efecto bola de nieve</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>CUL · Cultura de innovación</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="C9" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="D9" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="28" t="n">
-        <v>21.2514060876285</v>
-      </c>
       <c r="F9" s="28" t="n">
-        <v>31.15971242356779</v>
-      </c>
-      <c r="G9" s="4" t="n">
+        <v>21.25140608762847</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>31.15971242356774</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="I9" s="30" t="n">
         <v>-2</v>
       </c>
-      <c r="I9" s="21" t="n">
-        <v>3.67922000145532</v>
-      </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="21" t="n">
+        <v>3.679220001455313</v>
+      </c>
+      <c r="K9" s="13" t="n">
         <v>14.75783234768545</v>
       </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>Variable dependiente / de resultado</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Variable de resultado / dependiente</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>Falsa variable clave (espejismo); Nodo de efecto bola de nieve</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>EXP · Experiencia estudiantil</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="C10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="D10" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="28" t="n">
-        <v>14.56170975670292</v>
-      </c>
       <c r="F10" s="28" t="n">
-        <v>38.57789390494348</v>
-      </c>
-      <c r="G10" s="4" t="n">
+        <v>14.5617097567029</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>38.57789390494341</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H10" s="30" t="n">
+      <c r="I10" s="30" t="n">
         <v>-2</v>
       </c>
-      <c r="I10" s="21" t="n">
-        <v>2.14738170378525</v>
-      </c>
-      <c r="J10" s="13" t="n">
+      <c r="J10" s="21" t="n">
+        <v>2.147381703785245</v>
+      </c>
+      <c r="K10" s="13" t="n">
         <v>12.85157669322203</v>
       </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Variable dependiente / de resultado</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Variable de resultado / dependiente</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Variable de evolución regular</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>RES · Resistencia al cambio</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="C11" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="D11" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="28" t="n">
-        <v>19.97941608512383</v>
-      </c>
       <c r="F11" s="28" t="n">
-        <v>30.99871647522389</v>
-      </c>
-      <c r="G11" s="4" t="n">
+        <v>19.9794160851238</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>30.99871647522383</v>
+      </c>
+      <c r="H11" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="21" t="n">
-        <v>3.730493173481435</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>15.73389899047165</v>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>Variable dependiente / de resultado</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>3.730493173481429</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>15.73389899047163</v>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Variable de resultado / dependiente</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>Falsa variable clave (espejismo); Nodo de efecto bola de nieve</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>RET · Retención estudiantil</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="C12" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="D12" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="28" t="n">
-        <v>14.96589473882904</v>
-      </c>
       <c r="F12" s="28" t="n">
-        <v>23.19517771778834</v>
-      </c>
-      <c r="G12" s="4" t="n">
+        <v>14.96589473882901</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>23.1951777177883</v>
+      </c>
+      <c r="H12" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H12" s="29" t="n">
+      <c r="I12" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="21" t="n">
-        <v>1.437196761034053</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>8.761743242400676</v>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>Variable dependiente / de resultado</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="J12" s="21" t="n">
+        <v>1.437196761034049</v>
+      </c>
+      <c r="K12" s="13" t="n">
+        <v>8.761743242400666</v>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Variable de resultado / dependiente</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>Variable de evolución regular</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>NOR · Normativa y acreditación</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="C13" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="28" t="n">
-        <v>14.73114274800151</v>
-      </c>
       <c r="F13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4" t="n">
+        <v>14.73114274800148</v>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>1.110223024625157e-14</v>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Variable autónoma</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>Variable de evolución regular</t>
         </is>
@@ -5354,28 +5420,28 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1.46592057393983</v>
+        <v>1.465920573939827</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>4.517444987673217</v>
+        <v>4.517444987673213</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>3.317457839969312</v>
+        <v>3.317457839969307</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>8.545144406054764</v>
+        <v>8.545144406054753</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>8.23299312111682</v>
+        <v>8.232993121116809</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>7.398650684944265</v>
+        <v>7.39865068494425</v>
       </c>
       <c r="H5" s="22" t="n">
-        <v>8.071869749012141</v>
+        <v>8.071869749012128</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>3.865684240116183</v>
+        <v>3.865684240116175</v>
       </c>
       <c r="J5" s="22" t="n">
         <v>0</v>
@@ -5388,28 +5454,28 @@
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>1.125311645450641</v>
+        <v>1.125311645450639</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>1.418498526558171</v>
+        <v>1.418498526558168</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>3.83056331145824</v>
+        <v>3.830563311458238</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>4.70709450976613</v>
+        <v>4.707094509766124</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>3.162479642218536</v>
+        <v>3.162479642218531</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>5.549000782052843</v>
+        <v>5.549000782052835</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>3.019266511483517</v>
+        <v>3.019266511483511</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>3.085623772405527</v>
+        <v>3.085623772405521</v>
       </c>
       <c r="J6" s="22" t="n">
         <v>0</v>
@@ -5422,28 +5488,28 @@
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>1.230029073737875</v>
+        <v>1.230029073737873</v>
       </c>
       <c r="C7" s="22" t="n">
-        <v>1.627893562063615</v>
+        <v>1.627893562063612</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>1.170937222634377</v>
+        <v>1.170937222634375</v>
       </c>
       <c r="E7" s="22" t="n">
-        <v>3.567527476732368</v>
+        <v>3.567527476732362</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>3.238396263360756</v>
+        <v>3.23839626336075</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>5.772308299762903</v>
+        <v>5.772308299762896</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>2.748846215015519</v>
+        <v>2.748846215015513</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>3.637934584367535</v>
+        <v>3.63793458436753</v>
       </c>
       <c r="J7" s="22" t="n">
         <v>0</v>
@@ -5456,28 +5522,28 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>1.201259849953459</v>
+        <v>1.201259849953457</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>1.444109972427171</v>
+        <v>1.444109972427168</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>1.477898581735794</v>
+        <v>1.477898581735791</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>3.958993217981114</v>
+        <v>3.958993217981105</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>4.979192122467872</v>
+        <v>4.979192122467865</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>6.189039294874076</v>
+        <v>6.189039294874068</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>5.301064994339096</v>
+        <v>5.301064994339087</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>3.053611843666471</v>
+        <v>3.053611843666466</v>
       </c>
       <c r="J8" s="22" t="n">
         <v>0</v>
@@ -5490,28 +5556,28 @@
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.9007613169109756</v>
+        <v>0.9007613169109734</v>
       </c>
       <c r="C9" s="22" t="n">
-        <v>1.090324157348167</v>
+        <v>1.090324157348164</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>1.38607168653306</v>
+        <v>1.386071686533057</v>
       </c>
       <c r="E9" s="22" t="n">
-        <v>5.182495336935358</v>
+        <v>5.182495336935351</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>3.67922000145532</v>
+        <v>3.679220001455313</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>4.612576755583421</v>
+        <v>4.612576755583413</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>5.763866655080418</v>
+        <v>5.763866655080411</v>
       </c>
       <c r="I9" s="22" t="n">
-        <v>2.315310179237102</v>
+        <v>2.315310179237097</v>
       </c>
       <c r="J9" s="22" t="n">
         <v>0</v>
@@ -5524,28 +5590,28 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>1.546575889290308</v>
+        <v>1.546575889290307</v>
       </c>
       <c r="C10" s="22" t="n">
-        <v>1.83883822134632</v>
+        <v>1.838838221346318</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>1.143188511217501</v>
+        <v>1.143188511217499</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>2.251542848926266</v>
+        <v>2.251542848926261</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>1.984907004061643</v>
+        <v>1.984907004061639</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>2.14738170378525</v>
+        <v>2.147381703785245</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>1.935137650324372</v>
+        <v>1.935137650324368</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>3.861519631536507</v>
+        <v>3.861519631536505</v>
       </c>
       <c r="J10" s="22" t="n">
         <v>0</v>
@@ -5558,28 +5624,28 @@
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>0.8201839968606749</v>
+        <v>0.8201839968606731</v>
       </c>
       <c r="C11" s="22" t="n">
-        <v>1.011061852673228</v>
+        <v>1.011061852673226</v>
       </c>
       <c r="D11" s="22" t="n">
-        <v>1.942481083255581</v>
+        <v>1.942481083255579</v>
       </c>
       <c r="E11" s="22" t="n">
-        <v>5.084298434472478</v>
+        <v>5.084298434472472</v>
       </c>
       <c r="F11" s="22" t="n">
-        <v>4.819820008568112</v>
+        <v>4.819820008568107</v>
       </c>
       <c r="G11" s="22" t="n">
-        <v>4.13077034747217</v>
+        <v>4.130770347472163</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>3.730493173481435</v>
+        <v>3.730493173481429</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>2.170800361821586</v>
+        <v>2.170800361821582</v>
       </c>
       <c r="J11" s="22" t="n">
         <v>0</v>
@@ -5592,28 +5658,28 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
-        <v>1.350660212375459</v>
+        <v>1.350660212375458</v>
       </c>
       <c r="C12" s="22" t="n">
-        <v>2.762512908244746</v>
+        <v>2.762512908244744</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>1.578515852913601</v>
+        <v>1.578515852913599</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>2.560024106145279</v>
+        <v>2.560024106145274</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>2.065875399448626</v>
+        <v>2.065875399448622</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>2.64659592953064</v>
+        <v>2.646595929530634</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>2.001710330170687</v>
+        <v>2.001710330170682</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>1.437196761034053</v>
+        <v>1.437196761034049</v>
       </c>
       <c r="J12" s="22" t="n">
         <v>0</v>
@@ -5626,28 +5692,28 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>1.194294847400352</v>
+        <v>1.194294847400351</v>
       </c>
       <c r="C13" s="22" t="n">
-        <v>1.720002305974274</v>
+        <v>1.720002305974272</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>1.122525008986613</v>
+        <v>1.122525008986611</v>
       </c>
       <c r="E13" s="22" t="n">
-        <v>2.377672438156123</v>
+        <v>2.377672438156118</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>2.676048862325422</v>
+        <v>2.676048862325418</v>
       </c>
       <c r="G13" s="22" t="n">
-        <v>2.278951810723158</v>
+        <v>2.278951810723153</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>2.156954369798139</v>
+        <v>2.156954369798135</v>
       </c>
       <c r="I13" s="22" t="n">
-        <v>1.20469310463743</v>
+        <v>1.204693104637427</v>
       </c>
       <c r="J13" s="20" t="inlineStr">
         <is>
@@ -5755,28 +5821,28 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1.46592057393983</v>
+        <v>1.465920573939827</v>
       </c>
       <c r="C5" s="21" t="n">
-        <v>4.517444987673217</v>
+        <v>4.517444987673213</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>3.317457839969312</v>
+        <v>3.317457839969307</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>8.545144406054764</v>
+        <v>8.545144406054753</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>8.23299312111682</v>
+        <v>8.232993121116809</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>7.398650684944265</v>
+        <v>7.39865068494425</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>-8.071869749012141</v>
+        <v>-8.071869749012128</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>3.865684240116183</v>
+        <v>3.865684240116175</v>
       </c>
       <c r="J5" s="22" t="n">
         <v>0</v>
@@ -5789,28 +5855,28 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>1.125311645450641</v>
+        <v>1.125311645450639</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>1.418498526558171</v>
+        <v>1.418498526558168</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>3.83056331145824</v>
+        <v>3.830563311458238</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>4.70709450976613</v>
+        <v>4.707094509766124</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>3.162479642218536</v>
+        <v>3.162479642218531</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>5.549000782052843</v>
+        <v>5.549000782052835</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>-3.019266511483517</v>
+        <v>-3.019266511483511</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>3.085623772405527</v>
+        <v>3.085623772405521</v>
       </c>
       <c r="J6" s="22" t="n">
         <v>0</v>
@@ -5823,28 +5889,28 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>1.230029073737875</v>
+        <v>1.230029073737873</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.627893562063615</v>
+        <v>1.627893562063612</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>1.170937222634377</v>
+        <v>1.170937222634375</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>3.567527476732368</v>
+        <v>3.567527476732362</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>3.238396263360756</v>
+        <v>3.23839626336075</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>5.772308299762903</v>
+        <v>5.772308299762896</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>-2.748846215015519</v>
+        <v>-2.748846215015513</v>
       </c>
       <c r="I7" s="21" t="n">
-        <v>3.637934584367535</v>
+        <v>3.63793458436753</v>
       </c>
       <c r="J7" s="22" t="n">
         <v>0</v>
@@ -5857,28 +5923,28 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>1.201259849953459</v>
+        <v>1.201259849953457</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>1.444109972427171</v>
+        <v>1.444109972427168</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>1.477898581735794</v>
+        <v>1.477898581735791</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>3.958993217981114</v>
+        <v>3.958993217981105</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>4.979192122467872</v>
+        <v>4.979192122467865</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>6.189039294874076</v>
+        <v>6.189039294874068</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>-5.301064994339096</v>
+        <v>-5.301064994339087</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>3.053611843666471</v>
+        <v>3.053611843666466</v>
       </c>
       <c r="J8" s="22" t="n">
         <v>0</v>
@@ -5891,28 +5957,28 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>0.9007613169109756</v>
+        <v>0.9007613169109734</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.090324157348167</v>
+        <v>1.090324157348164</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>1.38607168653306</v>
+        <v>1.386071686533057</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>5.182495336935358</v>
+        <v>5.182495336935351</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>3.67922000145532</v>
+        <v>3.679220001455313</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>4.612576755583421</v>
+        <v>4.612576755583413</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>-5.763866655080418</v>
+        <v>-5.763866655080411</v>
       </c>
       <c r="I9" s="21" t="n">
-        <v>2.315310179237102</v>
+        <v>2.315310179237097</v>
       </c>
       <c r="J9" s="22" t="n">
         <v>0</v>
@@ -5925,28 +5991,28 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>1.546575889290308</v>
+        <v>1.546575889290307</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>1.83883822134632</v>
+        <v>1.838838221346318</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>1.143188511217501</v>
+        <v>1.143188511217499</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>2.251542848926266</v>
+        <v>2.251542848926261</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>1.984907004061643</v>
+        <v>1.984907004061639</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>2.14738170378525</v>
+        <v>2.147381703785245</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>-1.935137650324372</v>
+        <v>-1.935137650324368</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>3.861519631536507</v>
+        <v>3.861519631536505</v>
       </c>
       <c r="J10" s="22" t="n">
         <v>0</v>
@@ -5959,28 +6025,28 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>-0.8201839968606749</v>
+        <v>-0.8201839968606731</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>-1.011061852673228</v>
+        <v>-1.011061852673226</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>-1.942481083255581</v>
+        <v>-1.942481083255579</v>
       </c>
       <c r="E11" s="23" t="n">
-        <v>-5.084298434472478</v>
+        <v>-5.084298434472472</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>-4.819820008568112</v>
+        <v>-4.819820008568107</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>-4.13077034747217</v>
+        <v>-4.130770347472163</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>3.730493173481435</v>
+        <v>3.730493173481429</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>-2.170800361821586</v>
+        <v>-2.170800361821582</v>
       </c>
       <c r="J11" s="22" t="n">
         <v>0</v>
@@ -5993,28 +6059,28 @@
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>1.350660212375459</v>
+        <v>1.350660212375458</v>
       </c>
       <c r="C12" s="21" t="n">
-        <v>2.762512908244746</v>
+        <v>2.762512908244744</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>1.578515852913601</v>
+        <v>1.578515852913599</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>2.560024106145279</v>
+        <v>2.560024106145274</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>2.065875399448626</v>
+        <v>2.065875399448622</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>2.64659592953064</v>
+        <v>2.646595929530634</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>-2.001710330170687</v>
+        <v>-2.001710330170682</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>1.437196761034053</v>
+        <v>1.437196761034049</v>
       </c>
       <c r="J12" s="22" t="n">
         <v>0</v>
@@ -6027,28 +6093,28 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1.194294847400352</v>
+        <v>1.194294847400351</v>
       </c>
       <c r="C13" s="21" t="n">
-        <v>1.720002305974274</v>
+        <v>1.720002305974272</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>1.122525008986613</v>
+        <v>1.122525008986611</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>2.377672438156123</v>
+        <v>2.377672438156118</v>
       </c>
       <c r="F13" s="21" t="n">
-        <v>2.676048862325422</v>
+        <v>2.676048862325418</v>
       </c>
       <c r="G13" s="21" t="n">
-        <v>2.278951810723158</v>
+        <v>2.278951810723153</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>-2.156954369798139</v>
+        <v>-2.156954369798135</v>
       </c>
       <c r="I13" s="21" t="n">
-        <v>1.20469310463743</v>
+        <v>1.204693104637427</v>
       </c>
       <c r="J13" s="20" t="inlineStr">
         <is>
@@ -6156,28 +6222,28 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1.46592057393983</v>
+        <v>1.465920573939827</v>
       </c>
       <c r="C5" s="21" t="n">
-        <v>1.802932733565338</v>
+        <v>1.802932733565334</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>3.317457839969312</v>
+        <v>3.317457839969307</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>6.9076828998988</v>
+        <v>6.90768289989879</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>5.776800861882874</v>
+        <v>5.776800861882863</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>7.398650684944265</v>
+        <v>7.39865068494425</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>-6.350453796162025</v>
+        <v>-6.350453796162013</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>3.865684240116183</v>
+        <v>3.865684240116175</v>
       </c>
       <c r="J5" s="22" t="n">
         <v>0</v>
@@ -6190,28 +6256,28 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>1.125311645450641</v>
+        <v>1.125311645450639</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>1.418498526558171</v>
+        <v>1.418498526558168</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>1.116051057350361</v>
+        <v>1.116051057350359</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>3.069633003610167</v>
+        <v>3.069633003610161</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>3.162479642218536</v>
+        <v>3.162479642218531</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>4.688292805627785</v>
+        <v>4.688292805627778</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>-3.019266511483517</v>
+        <v>-3.019266511483511</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>3.085623772405527</v>
+        <v>3.085623772405521</v>
       </c>
       <c r="J6" s="22" t="n">
         <v>0</v>
@@ -6224,28 +6290,28 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>1.230029073737875</v>
+        <v>1.230029073737873</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.627893562063615</v>
+        <v>1.627893562063612</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>1.170937222634377</v>
+        <v>1.170937222634375</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>2.706819500307311</v>
+        <v>2.706819500307304</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>2.459595480289351</v>
+        <v>2.459595480289345</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>2.918620026260761</v>
+        <v>2.918620026260754</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>-2.748846215015519</v>
+        <v>-2.748846215015513</v>
       </c>
       <c r="I7" s="21" t="n">
-        <v>2.819203831289554</v>
+        <v>2.819203831289549</v>
       </c>
       <c r="J7" s="22" t="n">
         <v>0</v>
@@ -6258,28 +6324,28 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>1.201259849953459</v>
+        <v>1.201259849953457</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>1.444109972427171</v>
+        <v>1.444109972427168</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>1.477898581735794</v>
+        <v>1.477898581735791</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>3.958993217981114</v>
+        <v>3.958993217981105</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>3.341730616311908</v>
+        <v>3.341730616311901</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>3.474527040766198</v>
+        <v>3.474527040766189</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>-3.57964904148898</v>
+        <v>-3.579649041488971</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>3.053611843666471</v>
+        <v>3.053611843666466</v>
       </c>
       <c r="J8" s="22" t="n">
         <v>0</v>
@@ -6292,28 +6358,28 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>0.9007613169109756</v>
+        <v>0.9007613169109734</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.090324157348167</v>
+        <v>1.090324157348164</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>1.38607168653306</v>
+        <v>1.386071686533057</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>3.545033830779395</v>
+        <v>3.545033830779388</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>3.67922000145532</v>
+        <v>3.679220001455313</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>3.751868779158364</v>
+        <v>3.751868779158356</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>-3.307674395846472</v>
+        <v>-3.307674395846465</v>
       </c>
       <c r="I9" s="21" t="n">
-        <v>2.315310179237102</v>
+        <v>2.315310179237097</v>
       </c>
       <c r="J9" s="22" t="n">
         <v>0</v>
@@ -6326,28 +6392,28 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>0.80575766860859</v>
+        <v>0.8057576686085887</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>1.83883822134632</v>
+        <v>1.838838221346318</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>1.143188511217501</v>
+        <v>1.143188511217499</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>2.251542848926266</v>
+        <v>2.251542848926261</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>1.984907004061643</v>
+        <v>1.984907004061639</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>2.14738170378525</v>
+        <v>2.147381703785245</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>-1.935137650324372</v>
+        <v>-1.935137650324368</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>1.147007377428629</v>
+        <v>1.147007377428626</v>
       </c>
       <c r="J10" s="22" t="n">
         <v>0</v>
@@ -6360,28 +6426,28 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>-0.8201839968606749</v>
+        <v>-0.8201839968606731</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>-1.011061852673228</v>
+        <v>-1.011061852673226</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>-1.037643665219621</v>
+        <v>-1.037643665219619</v>
       </c>
       <c r="E11" s="23" t="n">
-        <v>-3.274623598400559</v>
+        <v>-3.274623598400553</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>-3.098404055717997</v>
+        <v>-3.098404055717991</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>-4.13077034747217</v>
+        <v>-4.130770347472163</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>3.730493173481435</v>
+        <v>3.730493173481429</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>-2.170800361821586</v>
+        <v>-2.170800361821582</v>
       </c>
       <c r="J11" s="22" t="n">
         <v>0</v>
@@ -6394,28 +6460,28 @@
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>0.5319294592974771</v>
+        <v>0.5319294592974758</v>
       </c>
       <c r="C12" s="21" t="n">
-        <v>1.041096955394631</v>
+        <v>1.041096955394629</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>1.578515852913601</v>
+        <v>1.578515852913599</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>2.560024106145279</v>
+        <v>2.560024106145274</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>2.065875399448626</v>
+        <v>2.065875399448622</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>2.64659592953064</v>
+        <v>2.646595929530634</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>-2.001710330170687</v>
+        <v>-2.001710330170682</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>1.437196761034053</v>
+        <v>1.437196761034049</v>
       </c>
       <c r="J12" s="22" t="n">
         <v>0</v>
@@ -6428,28 +6494,28 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>0.453476626718634</v>
+        <v>0.4534766267186326</v>
       </c>
       <c r="C13" s="21" t="n">
-        <v>0.9012715528962917</v>
+        <v>0.9012715528962897</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>1.122525008986613</v>
+        <v>1.122525008986611</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>2.377672438156123</v>
+        <v>2.377672438156118</v>
       </c>
       <c r="F13" s="21" t="n">
-        <v>1.935230641643704</v>
+        <v>1.9352306416437</v>
       </c>
       <c r="G13" s="21" t="n">
-        <v>2.278951810723158</v>
+        <v>2.278951810723153</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>-2.156954369798139</v>
+        <v>-2.156954369798135</v>
       </c>
       <c r="I13" s="21" t="n">
-        <v>1.20469310463743</v>
+        <v>1.204693104637427</v>
       </c>
       <c r="J13" s="24" t="n">
         <v>0</v>
@@ -6498,7 +6564,7 @@
         </is>
       </c>
       <c r="C18" s="21" t="n">
-        <v>7.398650684944265</v>
+        <v>7.39865068494425</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -6518,7 +6584,7 @@
         </is>
       </c>
       <c r="C19" s="21" t="n">
-        <v>6.9076828998988</v>
+        <v>6.90768289989879</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -6538,7 +6604,7 @@
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>-6.350453796162025</v>
+        <v>-6.350453796162013</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -6558,7 +6624,7 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>5.776800861882874</v>
+        <v>5.776800861882863</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -6578,7 +6644,7 @@
         </is>
       </c>
       <c r="C22" s="21" t="n">
-        <v>4.688292805627785</v>
+        <v>4.688292805627778</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -6598,7 +6664,7 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>-4.13077034747217</v>
+        <v>-4.130770347472163</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -6618,7 +6684,7 @@
         </is>
       </c>
       <c r="C24" s="21" t="n">
-        <v>3.865684240116183</v>
+        <v>3.865684240116175</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -6638,7 +6704,7 @@
         </is>
       </c>
       <c r="C25" s="21" t="n">
-        <v>3.751868779158364</v>
+        <v>3.751868779158356</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -6658,7 +6724,7 @@
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>-3.57964904148898</v>
+        <v>-3.579649041488971</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -6678,7 +6744,7 @@
         </is>
       </c>
       <c r="C27" s="21" t="n">
-        <v>3.545033830779395</v>
+        <v>3.545033830779388</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -6698,7 +6764,7 @@
         </is>
       </c>
       <c r="C28" s="21" t="n">
-        <v>3.474527040766198</v>
+        <v>3.474527040766189</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -6718,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" s="21" t="n">
-        <v>3.341730616311908</v>
+        <v>3.341730616311901</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -6738,7 +6804,7 @@
         </is>
       </c>
       <c r="C30" s="21" t="n">
-        <v>3.317457839969312</v>
+        <v>3.317457839969307</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -6758,7 +6824,7 @@
         </is>
       </c>
       <c r="C31" s="23" t="n">
-        <v>-3.307674395846472</v>
+        <v>-3.307674395846465</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -6778,7 +6844,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>-3.274623598400559</v>
+        <v>-3.274623598400553</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -6798,7 +6864,7 @@
         </is>
       </c>
       <c r="C33" s="21" t="n">
-        <v>3.162479642218536</v>
+        <v>3.162479642218531</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -6818,7 +6884,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>-3.098404055717997</v>
+        <v>-3.098404055717991</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -6838,7 +6904,7 @@
         </is>
       </c>
       <c r="C35" s="21" t="n">
-        <v>3.085623772405527</v>
+        <v>3.085623772405521</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -6858,7 +6924,7 @@
         </is>
       </c>
       <c r="C36" s="21" t="n">
-        <v>3.069633003610167</v>
+        <v>3.069633003610161</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -6878,7 +6944,7 @@
         </is>
       </c>
       <c r="C37" s="21" t="n">
-        <v>3.053611843666471</v>
+        <v>3.053611843666466</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -6898,7 +6964,7 @@
         </is>
       </c>
       <c r="C38" s="23" t="n">
-        <v>-3.019266511483517</v>
+        <v>-3.019266511483511</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -6918,7 +6984,7 @@
         </is>
       </c>
       <c r="C39" s="21" t="n">
-        <v>2.918620026260761</v>
+        <v>2.918620026260754</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -6938,7 +7004,7 @@
         </is>
       </c>
       <c r="C40" s="21" t="n">
-        <v>2.819203831289554</v>
+        <v>2.819203831289549</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -6958,7 +7024,7 @@
         </is>
       </c>
       <c r="C41" s="23" t="n">
-        <v>-2.748846215015519</v>
+        <v>-2.748846215015513</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -6978,7 +7044,7 @@
         </is>
       </c>
       <c r="C42" s="21" t="n">
-        <v>2.706819500307311</v>
+        <v>2.706819500307304</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -6998,7 +7064,7 @@
         </is>
       </c>
       <c r="C43" s="21" t="n">
-        <v>2.64659592953064</v>
+        <v>2.646595929530634</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -7018,7 +7084,7 @@
         </is>
       </c>
       <c r="C44" s="21" t="n">
-        <v>2.560024106145279</v>
+        <v>2.560024106145274</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -7038,7 +7104,7 @@
         </is>
       </c>
       <c r="C45" s="21" t="n">
-        <v>2.459595480289351</v>
+        <v>2.459595480289345</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -7058,7 +7124,7 @@
         </is>
       </c>
       <c r="C46" s="21" t="n">
-        <v>2.377672438156123</v>
+        <v>2.377672438156118</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -7078,7 +7144,7 @@
         </is>
       </c>
       <c r="C47" s="21" t="n">
-        <v>2.315310179237102</v>
+        <v>2.315310179237097</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -7098,7 +7164,7 @@
         </is>
       </c>
       <c r="C48" s="21" t="n">
-        <v>2.278951810723158</v>
+        <v>2.278951810723153</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -7118,7 +7184,7 @@
         </is>
       </c>
       <c r="C49" s="21" t="n">
-        <v>2.251542848926266</v>
+        <v>2.251542848926261</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -7138,7 +7204,7 @@
         </is>
       </c>
       <c r="C50" s="23" t="n">
-        <v>-2.170800361821586</v>
+        <v>-2.170800361821582</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -7158,7 +7224,7 @@
         </is>
       </c>
       <c r="C51" s="23" t="n">
-        <v>-2.156954369798139</v>
+        <v>-2.156954369798135</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -7178,7 +7244,7 @@
         </is>
       </c>
       <c r="C52" s="21" t="n">
-        <v>2.065875399448626</v>
+        <v>2.065875399448622</v>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
@@ -7198,7 +7264,7 @@
         </is>
       </c>
       <c r="C53" s="23" t="n">
-        <v>-2.001710330170687</v>
+        <v>-2.001710330170682</v>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
@@ -7218,7 +7284,7 @@
         </is>
       </c>
       <c r="C54" s="21" t="n">
-        <v>1.984907004061643</v>
+        <v>1.984907004061639</v>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
@@ -7238,7 +7304,7 @@
         </is>
       </c>
       <c r="C55" s="21" t="n">
-        <v>1.935230641643704</v>
+        <v>1.9352306416437</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
@@ -7258,7 +7324,7 @@
         </is>
       </c>
       <c r="C56" s="23" t="n">
-        <v>-1.935137650324372</v>
+        <v>-1.935137650324368</v>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
@@ -7278,7 +7344,7 @@
         </is>
       </c>
       <c r="C57" s="21" t="n">
-        <v>1.83883822134632</v>
+        <v>1.838838221346318</v>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
@@ -7298,7 +7364,7 @@
         </is>
       </c>
       <c r="C58" s="21" t="n">
-        <v>1.802932733565338</v>
+        <v>1.802932733565334</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
@@ -7318,7 +7384,7 @@
         </is>
       </c>
       <c r="C59" s="21" t="n">
-        <v>1.627893562063615</v>
+        <v>1.627893562063612</v>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
@@ -7338,7 +7404,7 @@
         </is>
       </c>
       <c r="C60" s="21" t="n">
-        <v>1.578515852913601</v>
+        <v>1.578515852913599</v>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
@@ -7358,7 +7424,7 @@
         </is>
       </c>
       <c r="C61" s="21" t="n">
-        <v>1.477898581735794</v>
+        <v>1.477898581735791</v>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
@@ -7378,7 +7444,7 @@
         </is>
       </c>
       <c r="C62" s="21" t="n">
-        <v>1.444109972427171</v>
+        <v>1.444109972427168</v>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
@@ -7398,7 +7464,7 @@
         </is>
       </c>
       <c r="C63" s="21" t="n">
-        <v>1.38607168653306</v>
+        <v>1.386071686533057</v>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
@@ -7418,7 +7484,7 @@
         </is>
       </c>
       <c r="C64" s="21" t="n">
-        <v>1.230029073737875</v>
+        <v>1.230029073737873</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
@@ -7438,7 +7504,7 @@
         </is>
       </c>
       <c r="C65" s="21" t="n">
-        <v>1.20469310463743</v>
+        <v>1.204693104637427</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
@@ -7458,7 +7524,7 @@
         </is>
       </c>
       <c r="C66" s="21" t="n">
-        <v>1.201259849953459</v>
+        <v>1.201259849953457</v>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
@@ -7478,7 +7544,7 @@
         </is>
       </c>
       <c r="C67" s="21" t="n">
-        <v>1.147007377428629</v>
+        <v>1.147007377428626</v>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
@@ -7498,7 +7564,7 @@
         </is>
       </c>
       <c r="C68" s="21" t="n">
-        <v>1.143188511217501</v>
+        <v>1.143188511217499</v>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
@@ -7518,7 +7584,7 @@
         </is>
       </c>
       <c r="C69" s="21" t="n">
-        <v>1.125311645450641</v>
+        <v>1.125311645450639</v>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
@@ -7538,7 +7604,7 @@
         </is>
       </c>
       <c r="C70" s="21" t="n">
-        <v>1.122525008986613</v>
+        <v>1.122525008986611</v>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
@@ -7558,7 +7624,7 @@
         </is>
       </c>
       <c r="C71" s="21" t="n">
-        <v>1.116051057350361</v>
+        <v>1.116051057350359</v>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
@@ -7578,7 +7644,7 @@
         </is>
       </c>
       <c r="C72" s="21" t="n">
-        <v>1.090324157348167</v>
+        <v>1.090324157348164</v>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
@@ -7598,7 +7664,7 @@
         </is>
       </c>
       <c r="C73" s="21" t="n">
-        <v>1.041096955394631</v>
+        <v>1.041096955394629</v>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
@@ -7618,7 +7684,7 @@
         </is>
       </c>
       <c r="C74" s="23" t="n">
-        <v>-1.037643665219621</v>
+        <v>-1.037643665219619</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
@@ -7638,7 +7704,7 @@
         </is>
       </c>
       <c r="C75" s="23" t="n">
-        <v>-1.011061852673228</v>
+        <v>-1.011061852673226</v>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
@@ -7658,7 +7724,7 @@
         </is>
       </c>
       <c r="C76" s="21" t="n">
-        <v>0.9012715528962917</v>
+        <v>0.9012715528962897</v>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
@@ -7678,7 +7744,7 @@
         </is>
       </c>
       <c r="C77" s="21" t="n">
-        <v>0.9007613169109756</v>
+        <v>0.9007613169109734</v>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
@@ -7698,7 +7764,7 @@
         </is>
       </c>
       <c r="C78" s="23" t="n">
-        <v>-0.8201839968606749</v>
+        <v>-0.8201839968606731</v>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
@@ -7718,7 +7784,7 @@
         </is>
       </c>
       <c r="C79" s="21" t="n">
-        <v>0.80575766860859</v>
+        <v>0.8057576686085887</v>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
@@ -7738,7 +7804,7 @@
         </is>
       </c>
       <c r="C80" s="21" t="n">
-        <v>0.5319294592974771</v>
+        <v>0.5319294592974758</v>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
@@ -7758,7 +7824,7 @@
         </is>
       </c>
       <c r="C81" s="21" t="n">
-        <v>0.453476626718634</v>
+        <v>0.4534766267186326</v>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>

</xml_diff>